<commit_message>
Backup local cache state before Google Drive stateless rewrite
</commit_message>
<xml_diff>
--- a/src/assets/mapping.xlsx
+++ b/src/assets/mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\company project\automation\src\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9495FE0-1AC9-45BF-9A5D-486F3D5A746C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C071CC67-F33C-4410-A76D-F377EB147378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5556" yWindow="852" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="3" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="53">
   <si>
     <t>Beban pokok penjualan</t>
   </si>
@@ -85,9 +85,6 @@
     <t>Beban keuangan</t>
   </si>
   <si>
-    <t>…..</t>
-  </si>
-  <si>
     <t>Laba (Rugi) tahun berjalan</t>
   </si>
   <si>
@@ -166,9 +163,6 @@
     <t>X1</t>
   </si>
   <si>
-    <t>extract</t>
-  </si>
-  <si>
     <t>source operasi</t>
   </si>
   <si>
@@ -176,13 +170,28 @@
   </si>
   <si>
     <t>master uraian</t>
+  </si>
+  <si>
+    <t>X6</t>
+  </si>
+  <si>
+    <t>X7</t>
+  </si>
+  <si>
+    <t>X8</t>
+  </si>
+  <si>
+    <t>X9</t>
+  </si>
+  <si>
+    <t>X5-X6</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -223,6 +232,12 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -317,7 +332,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -344,17 +359,11 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" quotePrefix="1"/>
     <xf numFmtId="16" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
@@ -640,7 +649,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FBC8ED1-1B02-4284-9476-3B295657A52B}">
-  <dimension ref="B1:M22"/>
+  <dimension ref="B1:K22"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="8.88671875" style="1"/>
@@ -653,14 +662,14 @@
     <col min="12" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B1" s="16" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="2" spans="2:13" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B1" s="14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="2:11" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C2" s="6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>8</v>
@@ -669,34 +678,28 @@
         <v>7</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="2:13" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C3" s="6">
         <v>1</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="15"/>
+      <c r="H3" s="13"/>
       <c r="I3" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J3" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="K3" s="14" t="s">
+      <c r="J3" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="M3" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="2:13" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K3" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C4" s="6">
         <v>2</v>
       </c>
@@ -704,119 +707,121 @@
         <v>0</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="M4" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="2:13" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C5" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D5" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C6" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="I5" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="J5" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="L5" s="14"/>
-    </row>
-    <row r="6" spans="2:13" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C6" s="6" t="s">
-        <v>34</v>
-      </c>
       <c r="D6" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="J6" s="12" t="s">
         <v>30</v>
       </c>
+      <c r="J6" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="K6" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="2:13" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C7" s="6">
         <v>4</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J7" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="2:13" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C8" s="6">
         <v>5</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="I8" s="13"/>
-      <c r="J8" s="12" t="s">
         <v>23</v>
       </c>
+      <c r="I8" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J8" s="11" t="s">
+        <v>22</v>
+      </c>
       <c r="K8" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="2:13" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C9" s="6">
         <v>6</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="I9" s="11"/>
+        <v>20</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="J9" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="2:13" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C10" s="6">
         <v>7</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I10" s="7"/>
+      <c r="I10" s="10" t="s">
+        <v>50</v>
+      </c>
       <c r="J10" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="2:13" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:11" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C11" s="6" t="s">
         <v>17</v>
       </c>
@@ -826,12 +831,14 @@
       <c r="E11" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="I11" s="10"/>
+      <c r="I11" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="J11" s="9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="2:13" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:11" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C12" s="6" t="s">
         <v>14</v>
       </c>
@@ -842,14 +849,14 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="2:13" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:11" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D13" s="7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="2:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="15" spans="2:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="2:13" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="2:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="15" spans="2:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="2:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="17" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="19" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -857,6 +864,7 @@
     <row r="21" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="22" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>